<commit_message>
Upload Download Summary - 2026-10-07 01:32:14
</commit_message>
<xml_diff>
--- a/assets/Dataset_Details.xlsx
+++ b/assets/Dataset_Details.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="101">
   <si>
     <t>Dataset</t>
   </si>
@@ -52,6 +52,213 @@
     <t>Datasize_Size_MB</t>
   </si>
   <si>
+    <t>Accidents</t>
+  </si>
+  <si>
+    <t>Atherosclerosis</t>
+  </si>
+  <si>
+    <t>AustralianFootball</t>
+  </si>
+  <si>
+    <t>Biodegradability</t>
+  </si>
+  <si>
+    <t>Bupa</t>
+  </si>
+  <si>
+    <t>CORA</t>
+  </si>
+  <si>
+    <t>Carcinogenesis</t>
+  </si>
+  <si>
+    <t>Chess</t>
+  </si>
+  <si>
+    <t>Countries</t>
+  </si>
+  <si>
+    <t>DCG</t>
+  </si>
+  <si>
+    <t>Dunur</t>
+  </si>
+  <si>
+    <t>Elti</t>
+  </si>
+  <si>
+    <t>FNHK</t>
+  </si>
+  <si>
+    <t>Facebook</t>
+  </si>
+  <si>
+    <t>Hepatitis_std</t>
+  </si>
+  <si>
+    <t>Mesh</t>
+  </si>
+  <si>
+    <t>Mooney_Family</t>
+  </si>
+  <si>
+    <t>MuskSmall</t>
+  </si>
+  <si>
+    <t>NBA</t>
+  </si>
+  <si>
+    <t>NCAA</t>
+  </si>
+  <si>
+    <t>OMOP_CDM_dayz</t>
+  </si>
+  <si>
+    <t>PTE</t>
+  </si>
+  <si>
+    <t>Pima</t>
+  </si>
+  <si>
+    <t>PremierLeague</t>
+  </si>
+  <si>
+    <t>Pyrimidine</t>
+  </si>
+  <si>
+    <t>SAP</t>
+  </si>
+  <si>
+    <t>SAT</t>
+  </si>
+  <si>
+    <t>SalesDB</t>
+  </si>
+  <si>
+    <t>Same_gen</t>
+  </si>
+  <si>
+    <t>Student_loan</t>
+  </si>
+  <si>
+    <t>Toxicology</t>
+  </si>
+  <si>
+    <t>Triazine</t>
+  </si>
+  <si>
+    <t>TubePricing</t>
+  </si>
+  <si>
+    <t>UTube</t>
+  </si>
+  <si>
+    <t>UW_std</t>
+  </si>
+  <si>
+    <t>WebKP</t>
+  </si>
+  <si>
+    <t>airbnb-simplified</t>
+  </si>
+  <si>
+    <t>fake_hotels</t>
+  </si>
+  <si>
+    <t>fake_hotels_extended</t>
+  </si>
+  <si>
+    <t>financial</t>
+  </si>
+  <si>
+    <t>ftp</t>
+  </si>
+  <si>
+    <t>genes</t>
+  </si>
+  <si>
+    <t>got_families</t>
+  </si>
+  <si>
+    <t>imdb_MovieLens</t>
+  </si>
+  <si>
+    <t>imdb_ijs</t>
+  </si>
+  <si>
+    <t>imdb_small</t>
+  </si>
+  <si>
+    <t>legalActs</t>
+  </si>
+  <si>
+    <t>multi_table_ID_demo_dataset</t>
+  </si>
+  <si>
+    <t>mutagenesis</t>
+  </si>
+  <si>
+    <t>nations</t>
+  </si>
+  <si>
+    <t>restbase</t>
+  </si>
+  <si>
+    <t>trains</t>
+  </si>
+  <si>
+    <t>university</t>
+  </si>
+  <si>
+    <t>world</t>
+  </si>
+  <si>
+    <t>MovieLens</t>
+  </si>
+  <si>
+    <t>Telstra</t>
+  </si>
+  <si>
+    <t>instacart_marketbasket_ml</t>
+  </si>
+  <si>
+    <t>rel-amazon</t>
+  </si>
+  <si>
+    <t>rel-arxiv</t>
+  </si>
+  <si>
+    <t>rel-avito</t>
+  </si>
+  <si>
+    <t>rel-event</t>
+  </si>
+  <si>
+    <t>rel-f1</t>
+  </si>
+  <si>
+    <t>rel-hm</t>
+  </si>
+  <si>
+    <t>rel-ratebeer</t>
+  </si>
+  <si>
+    <t>rel-salt</t>
+  </si>
+  <si>
+    <t>rel-stack</t>
+  </si>
+  <si>
+    <t>rel-trial</t>
+  </si>
+  <si>
+    <t>rossmann</t>
+  </si>
+  <si>
+    <t>walmart</t>
+  </si>
+  <si>
     <t>adult</t>
   </si>
   <si>
@@ -79,217 +286,22 @@
     <t>news</t>
   </si>
   <si>
-    <t>Accidents</t>
-  </si>
-  <si>
-    <t>Atherosclerosis</t>
-  </si>
-  <si>
-    <t>AustralianFootball</t>
-  </si>
-  <si>
-    <t>Biodegradability</t>
-  </si>
-  <si>
-    <t>Bupa</t>
-  </si>
-  <si>
-    <t>CORA</t>
-  </si>
-  <si>
-    <t>Carcinogenesis</t>
-  </si>
-  <si>
-    <t>Chess</t>
-  </si>
-  <si>
-    <t>Countries</t>
-  </si>
-  <si>
-    <t>DCG</t>
-  </si>
-  <si>
-    <t>Dunur</t>
-  </si>
-  <si>
-    <t>Elti</t>
-  </si>
-  <si>
-    <t>FNHK</t>
-  </si>
-  <si>
-    <t>Facebook</t>
-  </si>
-  <si>
-    <t>Hepatitis_std</t>
-  </si>
-  <si>
-    <t>Mesh</t>
-  </si>
-  <si>
-    <t>Mooney_Family</t>
-  </si>
-  <si>
-    <t>MuskSmall</t>
-  </si>
-  <si>
-    <t>NBA</t>
-  </si>
-  <si>
-    <t>NCAA</t>
-  </si>
-  <si>
-    <t>OMOP_CDM_dayz</t>
-  </si>
-  <si>
-    <t>PTE</t>
-  </si>
-  <si>
-    <t>Pima</t>
-  </si>
-  <si>
-    <t>PremierLeague</t>
-  </si>
-  <si>
-    <t>Pyrimidine</t>
-  </si>
-  <si>
-    <t>SAP</t>
-  </si>
-  <si>
-    <t>SAT</t>
-  </si>
-  <si>
-    <t>SalesDB</t>
-  </si>
-  <si>
-    <t>Same_gen</t>
-  </si>
-  <si>
-    <t>Student_loan</t>
-  </si>
-  <si>
-    <t>Toxicology</t>
-  </si>
-  <si>
-    <t>Triazine</t>
-  </si>
-  <si>
-    <t>TubePricing</t>
-  </si>
-  <si>
-    <t>UTube</t>
-  </si>
-  <si>
-    <t>UW_std</t>
-  </si>
-  <si>
-    <t>WebKP</t>
-  </si>
-  <si>
-    <t>airbnb-simplified</t>
-  </si>
-  <si>
-    <t>fake_hotels</t>
-  </si>
-  <si>
-    <t>fake_hotels_extended</t>
-  </si>
-  <si>
-    <t>financial</t>
-  </si>
-  <si>
-    <t>ftp</t>
-  </si>
-  <si>
-    <t>genes</t>
-  </si>
-  <si>
-    <t>got_families</t>
-  </si>
-  <si>
-    <t>imdb_MovieLens</t>
-  </si>
-  <si>
-    <t>imdb_ijs</t>
-  </si>
-  <si>
-    <t>imdb_small</t>
-  </si>
-  <si>
-    <t>legalActs</t>
-  </si>
-  <si>
-    <t>multi_table_ID_demo_dataset</t>
-  </si>
-  <si>
-    <t>mutagenesis</t>
-  </si>
-  <si>
-    <t>nations</t>
-  </si>
-  <si>
-    <t>restbase</t>
-  </si>
-  <si>
-    <t>trains</t>
-  </si>
-  <si>
-    <t>university</t>
-  </si>
-  <si>
-    <t>world</t>
-  </si>
-  <si>
-    <t>MovieLens</t>
-  </si>
-  <si>
-    <t>Telstra</t>
-  </si>
-  <si>
-    <t>instacart_marketbasket_ml</t>
-  </si>
-  <si>
-    <t>rel-amazon</t>
-  </si>
-  <si>
-    <t>rel-arxiv</t>
-  </si>
-  <si>
-    <t>rel-avito</t>
-  </si>
-  <si>
-    <t>rel-event</t>
-  </si>
-  <si>
-    <t>rel-f1</t>
-  </si>
-  <si>
-    <t>rel-hm</t>
-  </si>
-  <si>
-    <t>rel-ratebeer</t>
-  </si>
-  <si>
-    <t>rel-salt</t>
-  </si>
-  <si>
-    <t>rel-stack</t>
-  </si>
-  <si>
-    <t>rel-trial</t>
-  </si>
-  <si>
-    <t>rossmann</t>
-  </si>
-  <si>
-    <t>walmart</t>
+    <t>multi_table</t>
   </si>
   <si>
     <t>single_table</t>
   </si>
   <si>
-    <t>multi_table</t>
+    <t>HSASynthesizer</t>
+  </si>
+  <si>
+    <t>ClavaDDPMSynthesizer</t>
+  </si>
+  <si>
+    <t>IndependentSynthesizer</t>
+  </si>
+  <si>
+    <t>HMASynthesizer</t>
   </si>
   <si>
     <t>RealTabFormerSynthesizer</t>
@@ -298,22 +310,7 @@
     <t>TabDDPMSynthesizer</t>
   </si>
   <si>
-    <t>TVAESynthesizer</t>
-  </si>
-  <si>
     <t>GaussianCopulaSynthesizer</t>
-  </si>
-  <si>
-    <t>HSASynthesizer</t>
-  </si>
-  <si>
-    <t>ClavaDDPMSynthesizer</t>
-  </si>
-  <si>
-    <t>IndependentSynthesizer</t>
-  </si>
-  <si>
-    <t>HMASynthesizer</t>
   </si>
   <si>
     <t>Public</t>
@@ -729,31 +726,31 @@
         <v>92</v>
       </c>
       <c r="D2">
-        <v>15</v>
+        <v>43</v>
       </c>
       <c r="E2">
-        <v>32561</v>
+        <v>1463093</v>
       </c>
       <c r="F2">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="G2">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="H2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I2">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L2">
-        <v>20.848</v>
+        <v>1029.07</v>
       </c>
     </row>
     <row r="3" spans="1:12">
@@ -764,34 +761,34 @@
         <v>90</v>
       </c>
       <c r="C3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D3">
-        <v>37</v>
+        <v>198</v>
       </c>
       <c r="E3">
-        <v>20000</v>
+        <v>12781</v>
       </c>
       <c r="F3">
-        <v>37</v>
+        <v>0</v>
       </c>
       <c r="G3">
-        <v>0</v>
+        <v>193</v>
       </c>
       <c r="H3">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I3">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L3">
-        <v>33.428</v>
+        <v>7.22</v>
       </c>
     </row>
     <row r="4" spans="1:12">
@@ -802,34 +799,34 @@
         <v>90</v>
       </c>
       <c r="C4" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="D4">
-        <v>41</v>
+        <v>78</v>
       </c>
       <c r="E4">
-        <v>299285</v>
+        <v>139179</v>
       </c>
       <c r="F4">
-        <v>29</v>
+        <v>12</v>
       </c>
       <c r="G4">
-        <v>12</v>
+        <v>57</v>
       </c>
       <c r="H4">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K4" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L4">
-        <v>647.349</v>
+        <v>57.799</v>
       </c>
     </row>
     <row r="5" spans="1:12">
@@ -843,31 +840,31 @@
         <v>93</v>
       </c>
       <c r="D5">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="E5">
-        <v>20000</v>
+        <v>21895</v>
       </c>
       <c r="F5">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="G5">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H5">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="I5">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K5" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L5">
-        <v>24.462</v>
+        <v>4.414</v>
       </c>
     </row>
     <row r="6" spans="1:12">
@@ -878,34 +875,34 @@
         <v>90</v>
       </c>
       <c r="C6" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D6">
-        <v>55</v>
+        <v>17</v>
       </c>
       <c r="E6">
-        <v>581012</v>
+        <v>2762</v>
       </c>
       <c r="F6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G6">
-        <v>54</v>
+        <v>7</v>
       </c>
       <c r="H6">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="I6">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="J6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L6">
-        <v>255.645</v>
+        <v>0.204</v>
       </c>
     </row>
     <row r="7" spans="1:12">
@@ -916,34 +913,34 @@
         <v>90</v>
       </c>
       <c r="C7" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="D7">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="E7">
-        <v>1000</v>
+        <v>57353</v>
       </c>
       <c r="F7">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="G7">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H7">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I7">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K7" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L7">
-        <v>0.444</v>
+        <v>8.178000000000001</v>
       </c>
     </row>
     <row r="8" spans="1:12">
@@ -954,34 +951,34 @@
         <v>90</v>
       </c>
       <c r="C8" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D8">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="E8">
-        <v>20000</v>
+        <v>27443</v>
       </c>
       <c r="F8">
-        <v>27</v>
+        <v>2</v>
       </c>
       <c r="G8">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H8">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="I8">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="J8">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K8" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L8">
-        <v>24.82</v>
+        <v>5.962</v>
       </c>
     </row>
     <row r="9" spans="1:12">
@@ -995,31 +992,31 @@
         <v>92</v>
       </c>
       <c r="D9">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="E9">
-        <v>494021</v>
+        <v>2052</v>
       </c>
       <c r="F9">
+        <v>39</v>
+      </c>
+      <c r="G9">
         <v>4</v>
       </c>
-      <c r="G9">
-        <v>37</v>
-      </c>
       <c r="H9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K9" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L9">
-        <v>266.086</v>
+        <v>1.762</v>
       </c>
     </row>
     <row r="10" spans="1:12">
@@ -1030,34 +1027,34 @@
         <v>90</v>
       </c>
       <c r="C10" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D10">
-        <v>59</v>
+        <v>68</v>
       </c>
       <c r="E10">
-        <v>39644</v>
+        <v>22318</v>
       </c>
       <c r="F10">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="G10">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="H10">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I10">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J10">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K10" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L10">
-        <v>18.712</v>
+        <v>17.769</v>
       </c>
     </row>
     <row r="11" spans="1:12">
@@ -1065,37 +1062,37 @@
         <v>21</v>
       </c>
       <c r="B11" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C11" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="D11">
-        <v>43</v>
+        <v>6</v>
       </c>
       <c r="E11">
-        <v>1463093</v>
+        <v>8258</v>
       </c>
       <c r="F11">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="G11">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="H11">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I11">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J11">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K11" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L11">
-        <v>1029.07</v>
+        <v>1.072</v>
       </c>
     </row>
     <row r="12" spans="1:12">
@@ -1103,37 +1100,37 @@
         <v>22</v>
       </c>
       <c r="B12" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C12" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D12">
-        <v>198</v>
+        <v>50</v>
       </c>
       <c r="E12">
-        <v>12781</v>
+        <v>440</v>
       </c>
       <c r="F12">
+        <v>1</v>
+      </c>
+      <c r="G12">
         <v>0</v>
       </c>
-      <c r="G12">
-        <v>193</v>
-      </c>
       <c r="H12">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="I12">
-        <v>3</v>
+        <v>34</v>
       </c>
       <c r="J12">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K12" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L12">
-        <v>7.22</v>
+        <v>0.08599999999999999</v>
       </c>
     </row>
     <row r="13" spans="1:12">
@@ -1141,37 +1138,37 @@
         <v>23</v>
       </c>
       <c r="B13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C13" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D13">
-        <v>78</v>
+        <v>32</v>
       </c>
       <c r="E13">
-        <v>139179</v>
+        <v>1352</v>
       </c>
       <c r="F13">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="G13">
-        <v>57</v>
+        <v>0</v>
       </c>
       <c r="H13">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="I13">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="J13">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K13" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L13">
-        <v>57.799</v>
+        <v>0.266</v>
       </c>
     </row>
     <row r="14" spans="1:12">
@@ -1179,37 +1176,37 @@
         <v>24</v>
       </c>
       <c r="B14" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C14" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="D14">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="E14">
-        <v>21895</v>
+        <v>2113275</v>
       </c>
       <c r="F14">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="G14">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="H14">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I14">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="J14">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K14" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L14">
-        <v>4.414</v>
+        <v>409.557</v>
       </c>
     </row>
     <row r="15" spans="1:12">
@@ -1217,37 +1214,37 @@
         <v>25</v>
       </c>
       <c r="B15" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C15" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="D15">
-        <v>17</v>
+        <v>266</v>
       </c>
       <c r="E15">
-        <v>2762</v>
+        <v>10173</v>
       </c>
       <c r="F15">
+        <v>262</v>
+      </c>
+      <c r="G15">
         <v>0</v>
       </c>
-      <c r="G15">
-        <v>7</v>
-      </c>
       <c r="H15">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="I15">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="J15">
         <v>2</v>
       </c>
       <c r="K15" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L15">
-        <v>0.204</v>
+        <v>1.94</v>
       </c>
     </row>
     <row r="16" spans="1:12">
@@ -1255,37 +1252,37 @@
         <v>26</v>
       </c>
       <c r="B16" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C16" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D16">
-        <v>10</v>
+        <v>29</v>
       </c>
       <c r="E16">
-        <v>57353</v>
+        <v>12927</v>
       </c>
       <c r="F16">
         <v>2</v>
       </c>
       <c r="G16">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="H16">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="I16">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J16">
         <v>2</v>
       </c>
       <c r="K16" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L16">
-        <v>8.178000000000001</v>
+        <v>1.043</v>
       </c>
     </row>
     <row r="17" spans="1:12">
@@ -1293,37 +1290,37 @@
         <v>27</v>
       </c>
       <c r="B17" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C17" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D17">
-        <v>23</v>
+        <v>41</v>
       </c>
       <c r="E17">
-        <v>27443</v>
+        <v>2700</v>
       </c>
       <c r="F17">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G17">
         <v>2</v>
       </c>
       <c r="H17">
-        <v>6</v>
+        <v>29</v>
       </c>
       <c r="I17">
-        <v>13</v>
+        <v>33</v>
       </c>
       <c r="J17">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K17" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L17">
-        <v>5.962</v>
+        <v>0.237</v>
       </c>
     </row>
     <row r="18" spans="1:12">
@@ -1331,37 +1328,37 @@
         <v>28</v>
       </c>
       <c r="B18" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C18" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D18">
-        <v>46</v>
+        <v>202</v>
       </c>
       <c r="E18">
-        <v>2052</v>
+        <v>4425</v>
       </c>
       <c r="F18">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="G18">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H18">
-        <v>2</v>
+        <v>68</v>
       </c>
       <c r="I18">
-        <v>1</v>
+        <v>189</v>
       </c>
       <c r="J18">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K18" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L18">
-        <v>1.762</v>
+        <v>0.829</v>
       </c>
     </row>
     <row r="19" spans="1:12">
@@ -1369,37 +1366,37 @@
         <v>29</v>
       </c>
       <c r="B19" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C19" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="D19">
-        <v>68</v>
+        <v>170</v>
       </c>
       <c r="E19">
-        <v>22318</v>
+        <v>568</v>
       </c>
       <c r="F19">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="G19">
-        <v>53</v>
+        <v>167</v>
       </c>
       <c r="H19">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I19">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J19">
         <v>2</v>
       </c>
       <c r="K19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L19">
-        <v>17.769</v>
+        <v>0.702</v>
       </c>
     </row>
     <row r="20" spans="1:12">
@@ -1407,37 +1404,37 @@
         <v>30</v>
       </c>
       <c r="B20" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C20" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="D20">
-        <v>6</v>
+        <v>33</v>
       </c>
       <c r="E20">
-        <v>8258</v>
+        <v>1219</v>
       </c>
       <c r="F20">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G20">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="H20">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I20">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="J20">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K20" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L20">
-        <v>1.072</v>
+        <v>0.222</v>
       </c>
     </row>
     <row r="21" spans="1:12">
@@ -1445,37 +1442,37 @@
         <v>31</v>
       </c>
       <c r="B21" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C21" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D21">
-        <v>50</v>
+        <v>112</v>
       </c>
       <c r="E21">
-        <v>440</v>
+        <v>202305</v>
       </c>
       <c r="F21">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="G21">
-        <v>0</v>
+        <v>72</v>
       </c>
       <c r="H21">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="I21">
-        <v>34</v>
+        <v>19</v>
       </c>
       <c r="J21">
         <v>3</v>
       </c>
       <c r="K21" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L21">
-        <v>0.08599999999999999</v>
+        <v>50.824</v>
       </c>
     </row>
     <row r="22" spans="1:12">
@@ -1483,37 +1480,37 @@
         <v>32</v>
       </c>
       <c r="B22" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C22" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D22">
-        <v>32</v>
+        <v>432</v>
       </c>
       <c r="E22">
-        <v>1352</v>
+        <v>39000</v>
       </c>
       <c r="F22">
-        <v>1</v>
+        <v>108</v>
       </c>
       <c r="G22">
-        <v>0</v>
+        <v>51</v>
       </c>
       <c r="H22">
-        <v>11</v>
+        <v>39</v>
       </c>
       <c r="I22">
-        <v>20</v>
+        <v>171</v>
       </c>
       <c r="J22">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="K22" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L22">
-        <v>0.266</v>
+        <v>26.461</v>
       </c>
     </row>
     <row r="23" spans="1:12">
@@ -1521,37 +1518,37 @@
         <v>33</v>
       </c>
       <c r="B23" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C23" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="D23">
-        <v>26</v>
+        <v>97</v>
       </c>
       <c r="E23">
-        <v>2113275</v>
+        <v>29850</v>
       </c>
       <c r="F23">
-        <v>7</v>
+        <v>25</v>
       </c>
       <c r="G23">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H23">
-        <v>3</v>
+        <v>38</v>
       </c>
       <c r="I23">
-        <v>2</v>
+        <v>39</v>
       </c>
       <c r="J23">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K23" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L23">
-        <v>409.557</v>
+        <v>5.806</v>
       </c>
     </row>
     <row r="24" spans="1:12">
@@ -1559,37 +1556,37 @@
         <v>34</v>
       </c>
       <c r="B24" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C24" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="D24">
-        <v>266</v>
+        <v>18</v>
       </c>
       <c r="E24">
-        <v>10173</v>
+        <v>6912</v>
       </c>
       <c r="F24">
-        <v>262</v>
+        <v>1</v>
       </c>
       <c r="G24">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="H24">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="I24">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="J24">
         <v>2</v>
       </c>
       <c r="K24" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L24">
-        <v>1.94</v>
+        <v>0.514</v>
       </c>
     </row>
     <row r="25" spans="1:12">
@@ -1597,37 +1594,37 @@
         <v>35</v>
       </c>
       <c r="B25" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C25" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D25">
-        <v>29</v>
+        <v>218</v>
       </c>
       <c r="E25">
-        <v>12927</v>
+        <v>11308</v>
       </c>
       <c r="F25">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G25">
-        <v>14</v>
+        <v>204</v>
       </c>
       <c r="H25">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="I25">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J25">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K25" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L25">
-        <v>1.043</v>
+        <v>19.145</v>
       </c>
     </row>
     <row r="26" spans="1:12">
@@ -1635,37 +1632,37 @@
         <v>36</v>
       </c>
       <c r="B26" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C26" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="D26">
-        <v>41</v>
+        <v>14</v>
       </c>
       <c r="E26">
-        <v>2700</v>
+        <v>296</v>
       </c>
       <c r="F26">
         <v>0</v>
       </c>
       <c r="G26">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="H26">
-        <v>29</v>
+        <v>2</v>
       </c>
       <c r="I26">
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="J26">
         <v>2</v>
       </c>
       <c r="K26" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L26">
-        <v>0.237</v>
+        <v>0.034</v>
       </c>
     </row>
     <row r="27" spans="1:12">
@@ -1673,37 +1670,37 @@
         <v>37</v>
       </c>
       <c r="B27" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C27" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D27">
-        <v>202</v>
+        <v>42</v>
       </c>
       <c r="E27">
-        <v>4425</v>
+        <v>3841029</v>
       </c>
       <c r="F27">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="G27">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="H27">
-        <v>68</v>
+        <v>4</v>
       </c>
       <c r="I27">
-        <v>189</v>
+        <v>3</v>
       </c>
       <c r="J27">
         <v>3</v>
       </c>
       <c r="K27" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L27">
-        <v>0.829</v>
+        <v>504.868</v>
       </c>
     </row>
     <row r="28" spans="1:12">
@@ -1711,37 +1708,37 @@
         <v>38</v>
       </c>
       <c r="B28" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C28" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="D28">
-        <v>170</v>
+        <v>70</v>
       </c>
       <c r="E28">
-        <v>568</v>
+        <v>19867</v>
       </c>
       <c r="F28">
+        <v>1</v>
+      </c>
+      <c r="G28">
         <v>0</v>
       </c>
-      <c r="G28">
-        <v>167</v>
-      </c>
       <c r="H28">
-        <v>2</v>
+        <v>36</v>
       </c>
       <c r="I28">
-        <v>1</v>
+        <v>65</v>
       </c>
       <c r="J28">
         <v>2</v>
       </c>
       <c r="K28" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L28">
-        <v>0.702</v>
+        <v>1.38</v>
       </c>
     </row>
     <row r="29" spans="1:12">
@@ -1749,37 +1746,37 @@
         <v>39</v>
       </c>
       <c r="B29" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C29" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="D29">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="E29">
-        <v>1219</v>
+        <v>6735507</v>
       </c>
       <c r="F29">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="G29">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="H29">
         <v>4</v>
       </c>
       <c r="I29">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J29">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K29" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L29">
-        <v>0.222</v>
+        <v>272.229</v>
       </c>
     </row>
     <row r="30" spans="1:12">
@@ -1787,37 +1784,37 @@
         <v>40</v>
       </c>
       <c r="B30" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C30" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D30">
-        <v>112</v>
+        <v>11</v>
       </c>
       <c r="E30">
-        <v>202305</v>
+        <v>1536</v>
       </c>
       <c r="F30">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="G30">
-        <v>72</v>
+        <v>0</v>
       </c>
       <c r="H30">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="I30">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="J30">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K30" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L30">
-        <v>50.824</v>
+        <v>0.302</v>
       </c>
     </row>
     <row r="31" spans="1:12">
@@ -1825,37 +1822,37 @@
         <v>41</v>
       </c>
       <c r="B31" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C31" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D31">
-        <v>432</v>
+        <v>16</v>
       </c>
       <c r="E31">
-        <v>39000</v>
+        <v>5288</v>
       </c>
       <c r="F31">
-        <v>108</v>
+        <v>2</v>
       </c>
       <c r="G31">
-        <v>51</v>
+        <v>2</v>
       </c>
       <c r="H31">
-        <v>39</v>
+        <v>10</v>
       </c>
       <c r="I31">
-        <v>171</v>
+        <v>9</v>
       </c>
       <c r="J31">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="K31" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L31">
-        <v>26.461</v>
+        <v>0.609</v>
       </c>
     </row>
     <row r="32" spans="1:12">
@@ -1863,37 +1860,37 @@
         <v>42</v>
       </c>
       <c r="B32" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C32" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D32">
-        <v>97</v>
+        <v>12</v>
       </c>
       <c r="E32">
-        <v>29850</v>
+        <v>36922</v>
       </c>
       <c r="F32">
-        <v>25</v>
+        <v>3</v>
       </c>
       <c r="G32">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H32">
-        <v>38</v>
+        <v>4</v>
       </c>
       <c r="I32">
-        <v>39</v>
+        <v>5</v>
       </c>
       <c r="J32">
         <v>3</v>
       </c>
       <c r="K32" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L32">
-        <v>5.806</v>
+        <v>8.368</v>
       </c>
     </row>
     <row r="33" spans="1:12">
@@ -1901,37 +1898,37 @@
         <v>43</v>
       </c>
       <c r="B33" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C33" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="D33">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="E33">
-        <v>6912</v>
+        <v>1302</v>
       </c>
       <c r="F33">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G33">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="H33">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="I33">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="J33">
         <v>2</v>
       </c>
       <c r="K33" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L33">
-        <v>0.514</v>
+        <v>0.179</v>
       </c>
     </row>
     <row r="34" spans="1:12">
@@ -1939,37 +1936,37 @@
         <v>44</v>
       </c>
       <c r="B34" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C34" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="D34">
-        <v>218</v>
+        <v>192</v>
       </c>
       <c r="E34">
-        <v>11308</v>
+        <v>154899</v>
       </c>
       <c r="F34">
-        <v>5</v>
+        <v>54</v>
       </c>
       <c r="G34">
-        <v>204</v>
+        <v>92</v>
       </c>
       <c r="H34">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="I34">
-        <v>5</v>
+        <v>39</v>
       </c>
       <c r="J34">
         <v>3</v>
       </c>
       <c r="K34" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L34">
-        <v>19.145</v>
+        <v>40.634</v>
       </c>
     </row>
     <row r="35" spans="1:12">
@@ -1977,23 +1974,23 @@
         <v>45</v>
       </c>
       <c r="B35" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C35" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="D35">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="E35">
-        <v>296</v>
+        <v>2735</v>
       </c>
       <c r="F35">
+        <v>5</v>
+      </c>
+      <c r="G35">
         <v>0</v>
       </c>
-      <c r="G35">
-        <v>11</v>
-      </c>
       <c r="H35">
         <v>2</v>
       </c>
@@ -2004,10 +2001,10 @@
         <v>2</v>
       </c>
       <c r="K35" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L35">
-        <v>0.034</v>
+        <v>0.6830000000000001</v>
       </c>
     </row>
     <row r="36" spans="1:12">
@@ -2015,37 +2012,37 @@
         <v>46</v>
       </c>
       <c r="B36" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C36" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D36">
-        <v>42</v>
+        <v>14</v>
       </c>
       <c r="E36">
-        <v>3841029</v>
+        <v>712</v>
       </c>
       <c r="F36">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="G36">
-        <v>27</v>
+        <v>2</v>
       </c>
       <c r="H36">
         <v>4</v>
       </c>
       <c r="I36">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J36">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K36" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L36">
-        <v>504.868</v>
+        <v>0.091</v>
       </c>
     </row>
     <row r="37" spans="1:12">
@@ -2053,37 +2050,37 @@
         <v>47</v>
       </c>
       <c r="B37" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C37" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D37">
-        <v>70</v>
+        <v>8</v>
       </c>
       <c r="E37">
-        <v>19867</v>
+        <v>81850</v>
       </c>
       <c r="F37">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G37">
         <v>0</v>
       </c>
       <c r="H37">
-        <v>36</v>
+        <v>3</v>
       </c>
       <c r="I37">
-        <v>65</v>
+        <v>3</v>
       </c>
       <c r="J37">
         <v>2</v>
       </c>
       <c r="K37" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L37">
-        <v>1.38</v>
+        <v>22.794</v>
       </c>
     </row>
     <row r="38" spans="1:12">
@@ -2091,37 +2088,37 @@
         <v>48</v>
       </c>
       <c r="B38" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C38" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="D38">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="E38">
-        <v>6735507</v>
+        <v>5751408</v>
       </c>
       <c r="F38">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="G38">
         <v>2</v>
       </c>
       <c r="H38">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I38">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J38">
         <v>2</v>
       </c>
       <c r="K38" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L38">
-        <v>272.229</v>
+        <v>2058.564</v>
       </c>
     </row>
     <row r="39" spans="1:12">
@@ -2129,37 +2126,37 @@
         <v>49</v>
       </c>
       <c r="B39" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C39" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D39">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="E39">
-        <v>1536</v>
+        <v>668</v>
       </c>
       <c r="F39">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G39">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H39">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I39">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="J39">
         <v>2</v>
       </c>
       <c r="K39" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L39">
-        <v>0.302</v>
+        <v>0.308</v>
       </c>
     </row>
     <row r="40" spans="1:12">
@@ -2167,37 +2164,37 @@
         <v>50</v>
       </c>
       <c r="B40" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C40" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D40">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="E40">
-        <v>5288</v>
+        <v>668</v>
       </c>
       <c r="F40">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G40">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H40">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="I40">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="J40">
         <v>2</v>
       </c>
       <c r="K40" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L40">
-        <v>0.609</v>
+        <v>0.42</v>
       </c>
     </row>
     <row r="41" spans="1:12">
@@ -2205,37 +2202,37 @@
         <v>51</v>
       </c>
       <c r="B41" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C41" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D41">
-        <v>12</v>
+        <v>55</v>
       </c>
       <c r="E41">
-        <v>36922</v>
+        <v>1079680</v>
       </c>
       <c r="F41">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="G41">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="H41">
+        <v>8</v>
+      </c>
+      <c r="I41">
+        <v>8</v>
+      </c>
+      <c r="J41">
         <v>4</v>
       </c>
-      <c r="I41">
-        <v>5</v>
-      </c>
-      <c r="J41">
-        <v>3</v>
-      </c>
       <c r="K41" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L41">
-        <v>8.368</v>
+        <v>336.452</v>
       </c>
     </row>
     <row r="42" spans="1:12">
@@ -2243,22 +2240,22 @@
         <v>52</v>
       </c>
       <c r="B42" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C42" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="D42">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="E42">
-        <v>1302</v>
+        <v>96491</v>
       </c>
       <c r="F42">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G42">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="H42">
         <v>2</v>
@@ -2270,10 +2267,10 @@
         <v>2</v>
       </c>
       <c r="K42" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L42">
-        <v>0.179</v>
+        <v>33.67</v>
       </c>
     </row>
     <row r="43" spans="1:12">
@@ -2281,37 +2278,37 @@
         <v>53</v>
       </c>
       <c r="B43" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C43" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="D43">
-        <v>192</v>
+        <v>16</v>
       </c>
       <c r="E43">
-        <v>154899</v>
+        <v>6118</v>
       </c>
       <c r="F43">
-        <v>54</v>
+        <v>9</v>
       </c>
       <c r="G43">
-        <v>92</v>
+        <v>2</v>
       </c>
       <c r="H43">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="I43">
-        <v>39</v>
+        <v>3</v>
       </c>
       <c r="J43">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K43" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L43">
-        <v>40.634</v>
+        <v>2.908</v>
       </c>
     </row>
     <row r="44" spans="1:12">
@@ -2319,37 +2316,37 @@
         <v>54</v>
       </c>
       <c r="B44" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C44" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="D44">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E44">
-        <v>2735</v>
+        <v>23</v>
       </c>
       <c r="F44">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G44">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H44">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I44">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J44">
         <v>2</v>
       </c>
       <c r="K44" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L44">
-        <v>0.6830000000000001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="45" spans="1:12">
@@ -2357,37 +2354,37 @@
         <v>55</v>
       </c>
       <c r="B45" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C45" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="D45">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="E45">
-        <v>712</v>
+        <v>1249411</v>
       </c>
       <c r="F45">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G45">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="H45">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="I45">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J45">
         <v>2</v>
       </c>
       <c r="K45" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L45">
-        <v>0.091</v>
+        <v>114.714</v>
       </c>
     </row>
     <row r="46" spans="1:12">
@@ -2395,37 +2392,37 @@
         <v>56</v>
       </c>
       <c r="B46" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C46" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="D46">
-        <v>8</v>
+        <v>25</v>
       </c>
       <c r="E46">
-        <v>81850</v>
+        <v>5647694</v>
       </c>
       <c r="F46">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="G46">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H46">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="I46">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J46">
         <v>2</v>
       </c>
       <c r="K46" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L46">
-        <v>22.794</v>
+        <v>857.134</v>
       </c>
     </row>
     <row r="47" spans="1:12">
@@ -2433,37 +2430,37 @@
         <v>57</v>
       </c>
       <c r="B47" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C47" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="D47">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="E47">
-        <v>5751408</v>
+        <v>4395</v>
       </c>
       <c r="F47">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="G47">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H47">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="I47">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="J47">
         <v>2</v>
       </c>
       <c r="K47" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L47">
-        <v>2058.564</v>
+        <v>0.772</v>
       </c>
     </row>
     <row r="48" spans="1:12">
@@ -2471,37 +2468,37 @@
         <v>58</v>
       </c>
       <c r="B48" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C48" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="D48">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="E48">
-        <v>668</v>
+        <v>1754397</v>
       </c>
       <c r="F48">
+        <v>18</v>
+      </c>
+      <c r="G48">
+        <v>8</v>
+      </c>
+      <c r="H48">
         <v>5</v>
       </c>
-      <c r="G48">
-        <v>3</v>
-      </c>
-      <c r="H48">
-        <v>2</v>
-      </c>
       <c r="I48">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="J48">
         <v>2</v>
       </c>
       <c r="K48" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L48">
-        <v>0.308</v>
+        <v>773.989</v>
       </c>
     </row>
     <row r="49" spans="1:12">
@@ -2509,37 +2506,37 @@
         <v>59</v>
       </c>
       <c r="B49" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C49" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D49">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="E49">
-        <v>668</v>
+        <v>11150</v>
       </c>
       <c r="F49">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G49">
         <v>3</v>
       </c>
       <c r="H49">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I49">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J49">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K49" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L49">
-        <v>0.42</v>
+        <v>2.596</v>
       </c>
     </row>
     <row r="50" spans="1:12">
@@ -2547,37 +2544,37 @@
         <v>60</v>
       </c>
       <c r="B50" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C50" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="D50">
-        <v>55</v>
+        <v>15</v>
       </c>
       <c r="E50">
-        <v>1079680</v>
+        <v>10324</v>
       </c>
       <c r="F50">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="G50">
-        <v>21</v>
+        <v>7</v>
       </c>
       <c r="H50">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="I50">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="J50">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K50" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L50">
-        <v>336.452</v>
+        <v>2.065</v>
       </c>
     </row>
     <row r="51" spans="1:12">
@@ -2585,37 +2582,37 @@
         <v>61</v>
       </c>
       <c r="B51" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C51" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="D51">
-        <v>11</v>
+        <v>119</v>
       </c>
       <c r="E51">
-        <v>96491</v>
+        <v>11004</v>
       </c>
       <c r="F51">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G51">
-        <v>1</v>
+        <v>112</v>
       </c>
       <c r="H51">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I51">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J51">
         <v>2</v>
       </c>
       <c r="K51" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L51">
-        <v>33.67</v>
+        <v>1.833</v>
       </c>
     </row>
     <row r="52" spans="1:12">
@@ -2623,19 +2620,19 @@
         <v>62</v>
       </c>
       <c r="B52" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C52" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D52">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="E52">
-        <v>6118</v>
+        <v>19297</v>
       </c>
       <c r="F52">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="G52">
         <v>2</v>
@@ -2647,13 +2644,13 @@
         <v>3</v>
       </c>
       <c r="J52">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K52" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L52">
-        <v>2.908</v>
+        <v>3.573</v>
       </c>
     </row>
     <row r="53" spans="1:12">
@@ -2661,37 +2658,37 @@
         <v>63</v>
       </c>
       <c r="B53" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C53" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="D53">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="E53">
-        <v>23</v>
+        <v>83</v>
       </c>
       <c r="F53">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G53">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H53">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I53">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J53">
         <v>2</v>
       </c>
       <c r="K53" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L53">
-        <v>0.002</v>
+        <v>0.024</v>
       </c>
     </row>
     <row r="54" spans="1:12">
@@ -2699,37 +2696,37 @@
         <v>64</v>
       </c>
       <c r="B54" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C54" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="D54">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="E54">
-        <v>1249411</v>
+        <v>171</v>
       </c>
       <c r="F54">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G54">
         <v>9</v>
       </c>
       <c r="H54">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="I54">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J54">
         <v>2</v>
       </c>
       <c r="K54" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L54">
-        <v>114.714</v>
+        <v>0.013</v>
       </c>
     </row>
     <row r="55" spans="1:12">
@@ -2737,37 +2734,37 @@
         <v>65</v>
       </c>
       <c r="B55" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C55" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="D55">
         <v>25</v>
       </c>
       <c r="E55">
-        <v>5647694</v>
+        <v>5302</v>
       </c>
       <c r="F55">
+        <v>11</v>
+      </c>
+      <c r="G55">
         <v>9</v>
       </c>
-      <c r="G55">
-        <v>3</v>
-      </c>
       <c r="H55">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="I55">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="J55">
         <v>2</v>
       </c>
       <c r="K55" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L55">
-        <v>857.134</v>
+        <v>1.266</v>
       </c>
     </row>
     <row r="56" spans="1:12">
@@ -2775,28 +2772,28 @@
         <v>66</v>
       </c>
       <c r="B56" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C56" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D56">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="E56">
-        <v>4395</v>
+        <v>32231279</v>
       </c>
       <c r="F56">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="G56">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H56">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I56">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J56">
         <v>2</v>
@@ -2805,7 +2802,7 @@
         <v>100</v>
       </c>
       <c r="L56">
-        <v>0.772</v>
+        <v>969.1849999999999</v>
       </c>
     </row>
     <row r="57" spans="1:12">
@@ -2813,28 +2810,28 @@
         <v>67</v>
       </c>
       <c r="B57" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C57" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="D57">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="E57">
-        <v>1754397</v>
+        <v>148021</v>
       </c>
       <c r="F57">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="G57">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="H57">
         <v>5</v>
       </c>
       <c r="I57">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J57">
         <v>2</v>
@@ -2843,7 +2840,7 @@
         <v>100</v>
       </c>
       <c r="L57">
-        <v>773.989</v>
+        <v>20.369</v>
       </c>
     </row>
     <row r="58" spans="1:12">
@@ -2851,28 +2848,28 @@
         <v>68</v>
       </c>
       <c r="B58" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C58" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D58">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="E58">
-        <v>11150</v>
+        <v>173933</v>
       </c>
       <c r="F58">
         <v>4</v>
       </c>
       <c r="G58">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H58">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I58">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J58">
         <v>3</v>
@@ -2881,7 +2878,7 @@
         <v>100</v>
       </c>
       <c r="L58">
-        <v>2.596</v>
+        <v>40.435</v>
       </c>
     </row>
     <row r="59" spans="1:12">
@@ -2889,37 +2886,37 @@
         <v>69</v>
       </c>
       <c r="B59" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C59" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="D59">
         <v>15</v>
       </c>
       <c r="E59">
-        <v>10324</v>
+        <v>15000713</v>
       </c>
       <c r="F59">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G59">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="H59">
         <v>3</v>
       </c>
       <c r="I59">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J59">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K59" t="s">
         <v>100</v>
       </c>
       <c r="L59">
-        <v>2.065</v>
+        <v>10786.244</v>
       </c>
     </row>
     <row r="60" spans="1:12">
@@ -2927,28 +2924,28 @@
         <v>70</v>
       </c>
       <c r="B60" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C60" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="D60">
-        <v>119</v>
+        <v>21</v>
       </c>
       <c r="E60">
-        <v>11004</v>
+        <v>2146112</v>
       </c>
       <c r="F60">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G60">
-        <v>112</v>
+        <v>0</v>
       </c>
       <c r="H60">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="I60">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J60">
         <v>2</v>
@@ -2957,7 +2954,7 @@
         <v>100</v>
       </c>
       <c r="L60">
-        <v>1.833</v>
+        <v>523.1</v>
       </c>
     </row>
     <row r="61" spans="1:12">
@@ -2965,28 +2962,28 @@
         <v>71</v>
       </c>
       <c r="B61" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C61" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="D61">
-        <v>12</v>
+        <v>42</v>
       </c>
       <c r="E61">
-        <v>19297</v>
+        <v>20679117</v>
       </c>
       <c r="F61">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G61">
         <v>2</v>
       </c>
       <c r="H61">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="I61">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="J61">
         <v>3</v>
@@ -2995,7 +2992,7 @@
         <v>100</v>
       </c>
       <c r="L61">
-        <v>3.573</v>
+        <v>2754.622</v>
       </c>
     </row>
     <row r="62" spans="1:12">
@@ -3003,37 +3000,37 @@
         <v>72</v>
       </c>
       <c r="B62" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C62" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="D62">
-        <v>13</v>
+        <v>129</v>
       </c>
       <c r="E62">
-        <v>83</v>
+        <v>41328337</v>
       </c>
       <c r="F62">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="G62">
-        <v>4</v>
+        <v>102</v>
       </c>
       <c r="H62">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="I62">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="J62">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K62" t="s">
         <v>100</v>
       </c>
       <c r="L62">
-        <v>0.024</v>
+        <v>4578.511</v>
       </c>
     </row>
     <row r="63" spans="1:12">
@@ -3041,37 +3038,37 @@
         <v>73</v>
       </c>
       <c r="B63" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C63" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D63">
-        <v>19</v>
+        <v>67</v>
       </c>
       <c r="E63">
-        <v>171</v>
+        <v>74063</v>
       </c>
       <c r="F63">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G63">
+        <v>21</v>
+      </c>
+      <c r="H63">
         <v>9</v>
       </c>
-      <c r="H63">
-        <v>5</v>
-      </c>
       <c r="I63">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="J63">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K63" t="s">
         <v>100</v>
       </c>
       <c r="L63">
-        <v>0.013</v>
+        <v>10.695</v>
       </c>
     </row>
     <row r="64" spans="1:12">
@@ -3079,22 +3076,22 @@
         <v>74</v>
       </c>
       <c r="B64" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C64" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="D64">
-        <v>25</v>
+        <v>37</v>
       </c>
       <c r="E64">
-        <v>5302</v>
+        <v>16664809</v>
       </c>
       <c r="F64">
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="G64">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="H64">
         <v>3</v>
@@ -3109,7 +3106,7 @@
         <v>100</v>
       </c>
       <c r="L64">
-        <v>1.266</v>
+        <v>2008.983</v>
       </c>
     </row>
     <row r="65" spans="1:12">
@@ -3117,37 +3114,37 @@
         <v>75</v>
       </c>
       <c r="B65" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C65" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="D65">
-        <v>19</v>
+        <v>221</v>
       </c>
       <c r="E65">
-        <v>32231279</v>
+        <v>13787005</v>
       </c>
       <c r="F65">
-        <v>4</v>
+        <v>69</v>
       </c>
       <c r="G65">
-        <v>2</v>
+        <v>40</v>
       </c>
       <c r="H65">
+        <v>13</v>
+      </c>
+      <c r="I65">
+        <v>21</v>
+      </c>
+      <c r="J65">
         <v>6</v>
       </c>
-      <c r="I65">
-        <v>5</v>
-      </c>
-      <c r="J65">
-        <v>2</v>
-      </c>
       <c r="K65" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="L65">
-        <v>969.1849999999999</v>
+        <v>9343.481</v>
       </c>
     </row>
     <row r="66" spans="1:12">
@@ -3155,37 +3152,37 @@
         <v>76</v>
       </c>
       <c r="B66" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C66" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="D66">
-        <v>15</v>
+        <v>31</v>
       </c>
       <c r="E66">
-        <v>148021</v>
+        <v>4257145</v>
       </c>
       <c r="F66">
-        <v>5</v>
+        <v>17</v>
       </c>
       <c r="G66">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H66">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I66">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J66">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K66" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="L66">
-        <v>20.369</v>
+        <v>748.396</v>
       </c>
     </row>
     <row r="67" spans="1:12">
@@ -3193,37 +3190,37 @@
         <v>77</v>
       </c>
       <c r="B67" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C67" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="D67">
-        <v>12</v>
+        <v>51</v>
       </c>
       <c r="E67">
-        <v>173933</v>
+        <v>4247264</v>
       </c>
       <c r="F67">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="G67">
         <v>0</v>
       </c>
       <c r="H67">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="I67">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="J67">
         <v>3</v>
       </c>
       <c r="K67" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="L67">
-        <v>40.435</v>
+        <v>2679.668</v>
       </c>
     </row>
     <row r="68" spans="1:12">
@@ -3231,37 +3228,37 @@
         <v>78</v>
       </c>
       <c r="B68" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C68" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="D68">
+        <v>140</v>
+      </c>
+      <c r="E68">
+        <v>5434924</v>
+      </c>
+      <c r="F68">
+        <v>51</v>
+      </c>
+      <c r="G68">
         <v>15</v>
       </c>
-      <c r="E68">
-        <v>15000713</v>
-      </c>
-      <c r="F68">
-        <v>4</v>
-      </c>
-      <c r="G68">
-        <v>1</v>
-      </c>
       <c r="H68">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="I68">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="J68">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K68" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="L68">
-        <v>10786.244</v>
+        <v>3006.228</v>
       </c>
     </row>
     <row r="69" spans="1:12">
@@ -3269,37 +3266,37 @@
         <v>79</v>
       </c>
       <c r="B69" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C69" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="D69">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E69">
-        <v>2146112</v>
+        <v>1018324</v>
       </c>
       <c r="F69">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G69">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H69">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="I69">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="J69">
         <v>2</v>
       </c>
       <c r="K69" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="L69">
-        <v>523.1</v>
+        <v>184.365</v>
       </c>
     </row>
     <row r="70" spans="1:12">
@@ -3307,37 +3304,37 @@
         <v>80</v>
       </c>
       <c r="B70" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C70" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="D70">
-        <v>42</v>
+        <v>20</v>
       </c>
       <c r="E70">
-        <v>20679117</v>
+        <v>429805</v>
       </c>
       <c r="F70">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="G70">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="H70">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="I70">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="J70">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K70" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="L70">
-        <v>2754.622</v>
+        <v>40</v>
       </c>
     </row>
     <row r="71" spans="1:12">
@@ -3348,34 +3345,34 @@
         <v>91</v>
       </c>
       <c r="C71" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D71">
-        <v>129</v>
+        <v>15</v>
       </c>
       <c r="E71">
-        <v>41328337</v>
+        <v>32561</v>
       </c>
       <c r="F71">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G71">
-        <v>102</v>
+        <v>6</v>
       </c>
       <c r="H71">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="I71">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="J71">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K71" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="L71">
-        <v>4578.511</v>
+        <v>20.848</v>
       </c>
     </row>
     <row r="72" spans="1:12">
@@ -3386,34 +3383,34 @@
         <v>91</v>
       </c>
       <c r="C72" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D72">
-        <v>67</v>
+        <v>37</v>
       </c>
       <c r="E72">
-        <v>74063</v>
+        <v>20000</v>
       </c>
       <c r="F72">
-        <v>4</v>
+        <v>37</v>
       </c>
       <c r="G72">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="H72">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="I72">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="J72">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K72" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="L72">
-        <v>10.695</v>
+        <v>33.428</v>
       </c>
     </row>
     <row r="73" spans="1:12">
@@ -3424,34 +3421,34 @@
         <v>91</v>
       </c>
       <c r="C73" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="D73">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="E73">
-        <v>16664809</v>
+        <v>299285</v>
       </c>
       <c r="F73">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="G73">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="H73">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I73">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J73">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K73" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="L73">
-        <v>2008.983</v>
+        <v>647.349</v>
       </c>
     </row>
     <row r="74" spans="1:12">
@@ -3465,31 +3462,31 @@
         <v>97</v>
       </c>
       <c r="D74">
-        <v>221</v>
+        <v>20</v>
       </c>
       <c r="E74">
-        <v>13787005</v>
+        <v>20000</v>
       </c>
       <c r="F74">
-        <v>69</v>
+        <v>20</v>
       </c>
       <c r="G74">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="H74">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="I74">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="J74">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="K74" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="L74">
-        <v>9343.481</v>
+        <v>24.462</v>
       </c>
     </row>
     <row r="75" spans="1:12">
@@ -3500,34 +3497,34 @@
         <v>91</v>
       </c>
       <c r="C75" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="D75">
-        <v>31</v>
+        <v>55</v>
       </c>
       <c r="E75">
-        <v>4257145</v>
+        <v>581012</v>
       </c>
       <c r="F75">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="G75">
+        <v>54</v>
+      </c>
+      <c r="H75">
+        <v>1</v>
+      </c>
+      <c r="I75">
         <v>0</v>
       </c>
-      <c r="H75">
-        <v>4</v>
-      </c>
-      <c r="I75">
-        <v>6</v>
-      </c>
       <c r="J75">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K75" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="L75">
-        <v>748.396</v>
+        <v>255.645</v>
       </c>
     </row>
     <row r="76" spans="1:12">
@@ -3538,34 +3535,34 @@
         <v>91</v>
       </c>
       <c r="C76" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D76">
-        <v>51</v>
+        <v>25</v>
       </c>
       <c r="E76">
-        <v>4247264</v>
+        <v>1000</v>
       </c>
       <c r="F76">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="G76">
+        <v>5</v>
+      </c>
+      <c r="H76">
+        <v>1</v>
+      </c>
+      <c r="I76">
         <v>0</v>
       </c>
-      <c r="H76">
-        <v>7</v>
-      </c>
-      <c r="I76">
-        <v>10</v>
-      </c>
       <c r="J76">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K76" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="L76">
-        <v>2679.668</v>
+        <v>0.444</v>
       </c>
     </row>
     <row r="77" spans="1:12">
@@ -3576,34 +3573,34 @@
         <v>91</v>
       </c>
       <c r="C77" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D77">
-        <v>140</v>
+        <v>27</v>
       </c>
       <c r="E77">
-        <v>5434924</v>
+        <v>20000</v>
       </c>
       <c r="F77">
-        <v>51</v>
+        <v>27</v>
       </c>
       <c r="G77">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="H77">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="I77">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="J77">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K77" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="L77">
-        <v>3006.228</v>
+        <v>24.82</v>
       </c>
     </row>
     <row r="78" spans="1:12">
@@ -3614,34 +3611,34 @@
         <v>91</v>
       </c>
       <c r="C78" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D78">
-        <v>19</v>
+        <v>41</v>
       </c>
       <c r="E78">
-        <v>1018324</v>
+        <v>494021</v>
       </c>
       <c r="F78">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G78">
-        <v>10</v>
+        <v>37</v>
       </c>
       <c r="H78">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I78">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J78">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K78" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="L78">
-        <v>184.365</v>
+        <v>266.086</v>
       </c>
     </row>
     <row r="79" spans="1:12">
@@ -3652,34 +3649,34 @@
         <v>91</v>
       </c>
       <c r="C79" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D79">
-        <v>20</v>
+        <v>59</v>
       </c>
       <c r="E79">
-        <v>429805</v>
+        <v>39644</v>
       </c>
       <c r="F79">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G79">
-        <v>12</v>
+        <v>59</v>
       </c>
       <c r="H79">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I79">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J79">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K79" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="L79">
-        <v>40</v>
+        <v>18.712</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload Download Summary - 2026-10-11 01:34:52
</commit_message>
<xml_diff>
--- a/assets/Dataset_Details.xlsx
+++ b/assets/Dataset_Details.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="102">
   <si>
     <t>Dataset</t>
   </si>
@@ -52,6 +52,33 @@
     <t>Datasize_Size_MB</t>
   </si>
   <si>
+    <t>adult</t>
+  </si>
+  <si>
+    <t>alarm</t>
+  </si>
+  <si>
+    <t>census</t>
+  </si>
+  <si>
+    <t>child</t>
+  </si>
+  <si>
+    <t>covtype</t>
+  </si>
+  <si>
+    <t>expedia_hotel_logs</t>
+  </si>
+  <si>
+    <t>insurance</t>
+  </si>
+  <si>
+    <t>intrusion</t>
+  </si>
+  <si>
+    <t>news</t>
+  </si>
+  <si>
     <t>Accidents</t>
   </si>
   <si>
@@ -259,37 +286,19 @@
     <t>walmart</t>
   </si>
   <si>
-    <t>adult</t>
-  </si>
-  <si>
-    <t>alarm</t>
-  </si>
-  <si>
-    <t>census</t>
-  </si>
-  <si>
-    <t>child</t>
-  </si>
-  <si>
-    <t>covtype</t>
-  </si>
-  <si>
-    <t>expedia_hotel_logs</t>
-  </si>
-  <si>
-    <t>insurance</t>
-  </si>
-  <si>
-    <t>intrusion</t>
-  </si>
-  <si>
-    <t>news</t>
+    <t>single_table</t>
   </si>
   <si>
     <t>multi_table</t>
   </si>
   <si>
-    <t>single_table</t>
+    <t>RealTabFormerSynthesizer</t>
+  </si>
+  <si>
+    <t>TabDDPMSynthesizer</t>
+  </si>
+  <si>
+    <t>GaussianCopulaSynthesizer</t>
   </si>
   <si>
     <t>HSASynthesizer</t>
@@ -304,13 +313,7 @@
     <t>HMASynthesizer</t>
   </si>
   <si>
-    <t>RealTabFormerSynthesizer</t>
-  </si>
-  <si>
-    <t>TabDDPMSynthesizer</t>
-  </si>
-  <si>
-    <t>GaussianCopulaSynthesizer</t>
+    <t>MultiTableUniformSynthesizer</t>
   </si>
   <si>
     <t>Public</t>
@@ -726,31 +729,31 @@
         <v>92</v>
       </c>
       <c r="D2">
-        <v>43</v>
+        <v>15</v>
       </c>
       <c r="E2">
-        <v>1463093</v>
+        <v>32561</v>
       </c>
       <c r="F2">
-        <v>24</v>
+        <v>9</v>
       </c>
       <c r="G2">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="H2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I2">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L2">
-        <v>1029.07</v>
+        <v>20.848</v>
       </c>
     </row>
     <row r="3" spans="1:12">
@@ -761,34 +764,34 @@
         <v>90</v>
       </c>
       <c r="C3" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D3">
-        <v>198</v>
+        <v>37</v>
       </c>
       <c r="E3">
-        <v>12781</v>
+        <v>20000</v>
       </c>
       <c r="F3">
+        <v>37</v>
+      </c>
+      <c r="G3">
         <v>0</v>
       </c>
-      <c r="G3">
-        <v>193</v>
-      </c>
       <c r="H3">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I3">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L3">
-        <v>7.22</v>
+        <v>33.428</v>
       </c>
     </row>
     <row r="4" spans="1:12">
@@ -802,31 +805,31 @@
         <v>92</v>
       </c>
       <c r="D4">
-        <v>78</v>
+        <v>41</v>
       </c>
       <c r="E4">
-        <v>139179</v>
+        <v>299285</v>
       </c>
       <c r="F4">
+        <v>29</v>
+      </c>
+      <c r="G4">
         <v>12</v>
       </c>
-      <c r="G4">
-        <v>57</v>
-      </c>
       <c r="H4">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="J4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K4" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L4">
-        <v>57.799</v>
+        <v>647.349</v>
       </c>
     </row>
     <row r="5" spans="1:12">
@@ -840,31 +843,31 @@
         <v>93</v>
       </c>
       <c r="D5">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="E5">
-        <v>21895</v>
+        <v>20000</v>
       </c>
       <c r="F5">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="G5">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H5">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="I5">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="J5">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K5" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L5">
-        <v>4.414</v>
+        <v>24.462</v>
       </c>
     </row>
     <row r="6" spans="1:12">
@@ -875,34 +878,34 @@
         <v>90</v>
       </c>
       <c r="C6" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="D6">
-        <v>17</v>
+        <v>55</v>
       </c>
       <c r="E6">
-        <v>2762</v>
+        <v>581012</v>
       </c>
       <c r="F6">
+        <v>1</v>
+      </c>
+      <c r="G6">
+        <v>54</v>
+      </c>
+      <c r="H6">
+        <v>1</v>
+      </c>
+      <c r="I6">
         <v>0</v>
       </c>
-      <c r="G6">
-        <v>7</v>
-      </c>
-      <c r="H6">
-        <v>9</v>
-      </c>
-      <c r="I6">
-        <v>8</v>
-      </c>
       <c r="J6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K6" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L6">
-        <v>0.204</v>
+        <v>255.645</v>
       </c>
     </row>
     <row r="7" spans="1:12">
@@ -913,34 +916,34 @@
         <v>90</v>
       </c>
       <c r="C7" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D7">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="E7">
-        <v>57353</v>
+        <v>1000</v>
       </c>
       <c r="F7">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="G7">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H7">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I7">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K7" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L7">
-        <v>8.178000000000001</v>
+        <v>0.444</v>
       </c>
     </row>
     <row r="8" spans="1:12">
@@ -951,34 +954,34 @@
         <v>90</v>
       </c>
       <c r="C8" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D8">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="E8">
-        <v>27443</v>
+        <v>20000</v>
       </c>
       <c r="F8">
-        <v>2</v>
+        <v>27</v>
       </c>
       <c r="G8">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H8">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="I8">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="J8">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K8" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L8">
-        <v>5.962</v>
+        <v>24.82</v>
       </c>
     </row>
     <row r="9" spans="1:12">
@@ -992,31 +995,31 @@
         <v>92</v>
       </c>
       <c r="D9">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="E9">
-        <v>2052</v>
+        <v>494021</v>
       </c>
       <c r="F9">
-        <v>39</v>
+        <v>4</v>
       </c>
       <c r="G9">
-        <v>4</v>
+        <v>37</v>
       </c>
       <c r="H9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K9" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L9">
-        <v>1.762</v>
+        <v>266.086</v>
       </c>
     </row>
     <row r="10" spans="1:12">
@@ -1027,34 +1030,34 @@
         <v>90</v>
       </c>
       <c r="C10" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="D10">
-        <v>68</v>
+        <v>59</v>
       </c>
       <c r="E10">
-        <v>22318</v>
+        <v>39644</v>
       </c>
       <c r="F10">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="G10">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="H10">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I10">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J10">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K10" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L10">
-        <v>17.769</v>
+        <v>18.712</v>
       </c>
     </row>
     <row r="11" spans="1:12">
@@ -1062,37 +1065,37 @@
         <v>21</v>
       </c>
       <c r="B11" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C11" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D11">
-        <v>6</v>
+        <v>43</v>
       </c>
       <c r="E11">
-        <v>8258</v>
+        <v>1463093</v>
       </c>
       <c r="F11">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="G11">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="H11">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J11">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K11" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L11">
-        <v>1.072</v>
+        <v>1029.07</v>
       </c>
     </row>
     <row r="12" spans="1:12">
@@ -1100,37 +1103,37 @@
         <v>22</v>
       </c>
       <c r="B12" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C12" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="D12">
-        <v>50</v>
+        <v>198</v>
       </c>
       <c r="E12">
-        <v>440</v>
+        <v>12781</v>
       </c>
       <c r="F12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G12">
-        <v>0</v>
+        <v>193</v>
       </c>
       <c r="H12">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="I12">
-        <v>34</v>
+        <v>3</v>
       </c>
       <c r="J12">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K12" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L12">
-        <v>0.08599999999999999</v>
+        <v>7.22</v>
       </c>
     </row>
     <row r="13" spans="1:12">
@@ -1138,37 +1141,37 @@
         <v>23</v>
       </c>
       <c r="B13" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C13" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="D13">
-        <v>32</v>
+        <v>78</v>
       </c>
       <c r="E13">
-        <v>1352</v>
+        <v>139179</v>
       </c>
       <c r="F13">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="G13">
-        <v>0</v>
+        <v>57</v>
       </c>
       <c r="H13">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="I13">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="J13">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K13" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L13">
-        <v>0.266</v>
+        <v>57.799</v>
       </c>
     </row>
     <row r="14" spans="1:12">
@@ -1176,37 +1179,37 @@
         <v>24</v>
       </c>
       <c r="B14" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C14" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D14">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="E14">
-        <v>2113275</v>
+        <v>21895</v>
       </c>
       <c r="F14">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="G14">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="H14">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I14">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J14">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K14" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L14">
-        <v>409.557</v>
+        <v>4.414</v>
       </c>
     </row>
     <row r="15" spans="1:12">
@@ -1214,37 +1217,37 @@
         <v>25</v>
       </c>
       <c r="B15" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C15" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="D15">
-        <v>266</v>
+        <v>17</v>
       </c>
       <c r="E15">
-        <v>10173</v>
+        <v>2762</v>
       </c>
       <c r="F15">
-        <v>262</v>
+        <v>0</v>
       </c>
       <c r="G15">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="H15">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="I15">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="J15">
         <v>2</v>
       </c>
       <c r="K15" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L15">
-        <v>1.94</v>
+        <v>0.204</v>
       </c>
     </row>
     <row r="16" spans="1:12">
@@ -1252,37 +1255,37 @@
         <v>26</v>
       </c>
       <c r="B16" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C16" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="D16">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="E16">
-        <v>12927</v>
+        <v>57353</v>
       </c>
       <c r="F16">
         <v>2</v>
       </c>
       <c r="G16">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="H16">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="I16">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J16">
         <v>2</v>
       </c>
       <c r="K16" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L16">
-        <v>1.043</v>
+        <v>8.178000000000001</v>
       </c>
     </row>
     <row r="17" spans="1:12">
@@ -1290,37 +1293,37 @@
         <v>27</v>
       </c>
       <c r="B17" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C17" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="D17">
-        <v>41</v>
+        <v>23</v>
       </c>
       <c r="E17">
-        <v>2700</v>
+        <v>27443</v>
       </c>
       <c r="F17">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G17">
         <v>2</v>
       </c>
       <c r="H17">
-        <v>29</v>
+        <v>6</v>
       </c>
       <c r="I17">
-        <v>33</v>
+        <v>13</v>
       </c>
       <c r="J17">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K17" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L17">
-        <v>0.237</v>
+        <v>5.962</v>
       </c>
     </row>
     <row r="18" spans="1:12">
@@ -1328,37 +1331,37 @@
         <v>28</v>
       </c>
       <c r="B18" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C18" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="D18">
-        <v>202</v>
+        <v>46</v>
       </c>
       <c r="E18">
-        <v>4425</v>
+        <v>2052</v>
       </c>
       <c r="F18">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="G18">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H18">
-        <v>68</v>
+        <v>2</v>
       </c>
       <c r="I18">
-        <v>189</v>
+        <v>1</v>
       </c>
       <c r="J18">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K18" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L18">
-        <v>0.829</v>
+        <v>1.762</v>
       </c>
     </row>
     <row r="19" spans="1:12">
@@ -1366,37 +1369,37 @@
         <v>29</v>
       </c>
       <c r="B19" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C19" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D19">
-        <v>170</v>
+        <v>68</v>
       </c>
       <c r="E19">
-        <v>568</v>
+        <v>22318</v>
       </c>
       <c r="F19">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="G19">
-        <v>167</v>
+        <v>53</v>
       </c>
       <c r="H19">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I19">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J19">
         <v>2</v>
       </c>
       <c r="K19" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L19">
-        <v>0.702</v>
+        <v>17.769</v>
       </c>
     </row>
     <row r="20" spans="1:12">
@@ -1404,37 +1407,37 @@
         <v>30</v>
       </c>
       <c r="B20" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C20" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="D20">
-        <v>33</v>
+        <v>6</v>
       </c>
       <c r="E20">
-        <v>1219</v>
+        <v>8258</v>
       </c>
       <c r="F20">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G20">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="H20">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I20">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J20">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K20" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L20">
-        <v>0.222</v>
+        <v>1.072</v>
       </c>
     </row>
     <row r="21" spans="1:12">
@@ -1442,37 +1445,37 @@
         <v>31</v>
       </c>
       <c r="B21" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C21" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="D21">
-        <v>112</v>
+        <v>50</v>
       </c>
       <c r="E21">
-        <v>202305</v>
+        <v>440</v>
       </c>
       <c r="F21">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="G21">
-        <v>72</v>
+        <v>0</v>
       </c>
       <c r="H21">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="I21">
-        <v>19</v>
+        <v>34</v>
       </c>
       <c r="J21">
         <v>3</v>
       </c>
       <c r="K21" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L21">
-        <v>50.824</v>
+        <v>0.08599999999999999</v>
       </c>
     </row>
     <row r="22" spans="1:12">
@@ -1480,37 +1483,37 @@
         <v>32</v>
       </c>
       <c r="B22" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C22" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="D22">
-        <v>432</v>
+        <v>32</v>
       </c>
       <c r="E22">
-        <v>39000</v>
+        <v>1352</v>
       </c>
       <c r="F22">
-        <v>108</v>
+        <v>1</v>
       </c>
       <c r="G22">
-        <v>51</v>
+        <v>0</v>
       </c>
       <c r="H22">
-        <v>39</v>
+        <v>11</v>
       </c>
       <c r="I22">
-        <v>171</v>
+        <v>20</v>
       </c>
       <c r="J22">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="K22" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L22">
-        <v>26.461</v>
+        <v>0.266</v>
       </c>
     </row>
     <row r="23" spans="1:12">
@@ -1518,37 +1521,37 @@
         <v>33</v>
       </c>
       <c r="B23" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C23" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="D23">
-        <v>97</v>
+        <v>26</v>
       </c>
       <c r="E23">
-        <v>29850</v>
+        <v>2113275</v>
       </c>
       <c r="F23">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="G23">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H23">
-        <v>38</v>
+        <v>3</v>
       </c>
       <c r="I23">
-        <v>39</v>
+        <v>2</v>
       </c>
       <c r="J23">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K23" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L23">
-        <v>5.806</v>
+        <v>409.557</v>
       </c>
     </row>
     <row r="24" spans="1:12">
@@ -1556,37 +1559,37 @@
         <v>34</v>
       </c>
       <c r="B24" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C24" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D24">
-        <v>18</v>
+        <v>266</v>
       </c>
       <c r="E24">
-        <v>6912</v>
+        <v>10173</v>
       </c>
       <c r="F24">
-        <v>1</v>
+        <v>262</v>
       </c>
       <c r="G24">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="H24">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="I24">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="J24">
         <v>2</v>
       </c>
       <c r="K24" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L24">
-        <v>0.514</v>
+        <v>1.94</v>
       </c>
     </row>
     <row r="25" spans="1:12">
@@ -1594,37 +1597,37 @@
         <v>35</v>
       </c>
       <c r="B25" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C25" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="D25">
-        <v>218</v>
+        <v>29</v>
       </c>
       <c r="E25">
-        <v>11308</v>
+        <v>12927</v>
       </c>
       <c r="F25">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G25">
-        <v>204</v>
+        <v>14</v>
       </c>
       <c r="H25">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="I25">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J25">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K25" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L25">
-        <v>19.145</v>
+        <v>1.043</v>
       </c>
     </row>
     <row r="26" spans="1:12">
@@ -1632,37 +1635,37 @@
         <v>36</v>
       </c>
       <c r="B26" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C26" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D26">
-        <v>14</v>
+        <v>41</v>
       </c>
       <c r="E26">
-        <v>296</v>
+        <v>2700</v>
       </c>
       <c r="F26">
         <v>0</v>
       </c>
       <c r="G26">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="H26">
-        <v>2</v>
+        <v>29</v>
       </c>
       <c r="I26">
-        <v>1</v>
+        <v>33</v>
       </c>
       <c r="J26">
         <v>2</v>
       </c>
       <c r="K26" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L26">
-        <v>0.034</v>
+        <v>0.237</v>
       </c>
     </row>
     <row r="27" spans="1:12">
@@ -1670,37 +1673,37 @@
         <v>37</v>
       </c>
       <c r="B27" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C27" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="D27">
-        <v>42</v>
+        <v>202</v>
       </c>
       <c r="E27">
-        <v>3841029</v>
+        <v>4425</v>
       </c>
       <c r="F27">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="G27">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="H27">
-        <v>4</v>
+        <v>68</v>
       </c>
       <c r="I27">
-        <v>3</v>
+        <v>189</v>
       </c>
       <c r="J27">
         <v>3</v>
       </c>
       <c r="K27" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L27">
-        <v>504.868</v>
+        <v>0.829</v>
       </c>
     </row>
     <row r="28" spans="1:12">
@@ -1708,37 +1711,37 @@
         <v>38</v>
       </c>
       <c r="B28" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C28" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="D28">
-        <v>70</v>
+        <v>170</v>
       </c>
       <c r="E28">
-        <v>19867</v>
+        <v>568</v>
       </c>
       <c r="F28">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G28">
-        <v>0</v>
+        <v>167</v>
       </c>
       <c r="H28">
-        <v>36</v>
+        <v>2</v>
       </c>
       <c r="I28">
-        <v>65</v>
+        <v>1</v>
       </c>
       <c r="J28">
         <v>2</v>
       </c>
       <c r="K28" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L28">
-        <v>1.38</v>
+        <v>0.702</v>
       </c>
     </row>
     <row r="29" spans="1:12">
@@ -1746,37 +1749,37 @@
         <v>39</v>
       </c>
       <c r="B29" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C29" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D29">
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="E29">
-        <v>6735507</v>
+        <v>1219</v>
       </c>
       <c r="F29">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="G29">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="H29">
         <v>4</v>
       </c>
       <c r="I29">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J29">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K29" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L29">
-        <v>272.229</v>
+        <v>0.222</v>
       </c>
     </row>
     <row r="30" spans="1:12">
@@ -1784,37 +1787,37 @@
         <v>40</v>
       </c>
       <c r="B30" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C30" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="D30">
-        <v>11</v>
+        <v>112</v>
       </c>
       <c r="E30">
-        <v>1536</v>
+        <v>202305</v>
       </c>
       <c r="F30">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="G30">
-        <v>0</v>
+        <v>72</v>
       </c>
       <c r="H30">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="I30">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="J30">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K30" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L30">
-        <v>0.302</v>
+        <v>50.824</v>
       </c>
     </row>
     <row r="31" spans="1:12">
@@ -1822,37 +1825,37 @@
         <v>41</v>
       </c>
       <c r="B31" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C31" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="D31">
-        <v>16</v>
+        <v>432</v>
       </c>
       <c r="E31">
-        <v>5288</v>
+        <v>39000</v>
       </c>
       <c r="F31">
-        <v>2</v>
+        <v>108</v>
       </c>
       <c r="G31">
-        <v>2</v>
+        <v>51</v>
       </c>
       <c r="H31">
-        <v>10</v>
+        <v>39</v>
       </c>
       <c r="I31">
+        <v>171</v>
+      </c>
+      <c r="J31">
         <v>9</v>
       </c>
-      <c r="J31">
-        <v>2</v>
-      </c>
       <c r="K31" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L31">
-        <v>0.609</v>
+        <v>26.461</v>
       </c>
     </row>
     <row r="32" spans="1:12">
@@ -1860,37 +1863,37 @@
         <v>42</v>
       </c>
       <c r="B32" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C32" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="D32">
-        <v>12</v>
+        <v>97</v>
       </c>
       <c r="E32">
-        <v>36922</v>
+        <v>29850</v>
       </c>
       <c r="F32">
-        <v>3</v>
+        <v>25</v>
       </c>
       <c r="G32">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="H32">
-        <v>4</v>
+        <v>38</v>
       </c>
       <c r="I32">
-        <v>5</v>
+        <v>39</v>
       </c>
       <c r="J32">
         <v>3</v>
       </c>
       <c r="K32" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L32">
-        <v>8.368</v>
+        <v>5.806</v>
       </c>
     </row>
     <row r="33" spans="1:12">
@@ -1898,37 +1901,37 @@
         <v>43</v>
       </c>
       <c r="B33" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C33" t="s">
         <v>95</v>
       </c>
       <c r="D33">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="E33">
-        <v>1302</v>
+        <v>6912</v>
       </c>
       <c r="F33">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G33">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="H33">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="I33">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="J33">
         <v>2</v>
       </c>
       <c r="K33" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L33">
-        <v>0.179</v>
+        <v>0.514</v>
       </c>
     </row>
     <row r="34" spans="1:12">
@@ -1936,37 +1939,37 @@
         <v>44</v>
       </c>
       <c r="B34" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C34" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="D34">
-        <v>192</v>
+        <v>218</v>
       </c>
       <c r="E34">
-        <v>154899</v>
+        <v>11308</v>
       </c>
       <c r="F34">
-        <v>54</v>
+        <v>5</v>
       </c>
       <c r="G34">
-        <v>92</v>
+        <v>204</v>
       </c>
       <c r="H34">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="I34">
-        <v>39</v>
+        <v>5</v>
       </c>
       <c r="J34">
         <v>3</v>
       </c>
       <c r="K34" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L34">
-        <v>40.634</v>
+        <v>19.145</v>
       </c>
     </row>
     <row r="35" spans="1:12">
@@ -1974,22 +1977,22 @@
         <v>45</v>
       </c>
       <c r="B35" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C35" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="D35">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="E35">
-        <v>2735</v>
+        <v>296</v>
       </c>
       <c r="F35">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G35">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="H35">
         <v>2</v>
@@ -2001,10 +2004,10 @@
         <v>2</v>
       </c>
       <c r="K35" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L35">
-        <v>0.6830000000000001</v>
+        <v>0.034</v>
       </c>
     </row>
     <row r="36" spans="1:12">
@@ -2012,37 +2015,37 @@
         <v>46</v>
       </c>
       <c r="B36" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C36" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="D36">
-        <v>14</v>
+        <v>42</v>
       </c>
       <c r="E36">
-        <v>712</v>
+        <v>3841029</v>
       </c>
       <c r="F36">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="G36">
-        <v>2</v>
+        <v>27</v>
       </c>
       <c r="H36">
         <v>4</v>
       </c>
       <c r="I36">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J36">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K36" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L36">
-        <v>0.091</v>
+        <v>504.868</v>
       </c>
     </row>
     <row r="37" spans="1:12">
@@ -2050,37 +2053,37 @@
         <v>47</v>
       </c>
       <c r="B37" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C37" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="D37">
-        <v>8</v>
+        <v>70</v>
       </c>
       <c r="E37">
-        <v>81850</v>
+        <v>19867</v>
       </c>
       <c r="F37">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G37">
         <v>0</v>
       </c>
       <c r="H37">
-        <v>3</v>
+        <v>36</v>
       </c>
       <c r="I37">
-        <v>3</v>
+        <v>65</v>
       </c>
       <c r="J37">
         <v>2</v>
       </c>
       <c r="K37" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L37">
-        <v>22.794</v>
+        <v>1.38</v>
       </c>
     </row>
     <row r="38" spans="1:12">
@@ -2088,37 +2091,37 @@
         <v>48</v>
       </c>
       <c r="B38" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C38" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="D38">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="E38">
-        <v>5751408</v>
+        <v>6735507</v>
       </c>
       <c r="F38">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="G38">
         <v>2</v>
       </c>
       <c r="H38">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I38">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J38">
         <v>2</v>
       </c>
       <c r="K38" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L38">
-        <v>2058.564</v>
+        <v>272.229</v>
       </c>
     </row>
     <row r="39" spans="1:12">
@@ -2126,37 +2129,37 @@
         <v>49</v>
       </c>
       <c r="B39" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C39" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="D39">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="E39">
-        <v>668</v>
+        <v>1536</v>
       </c>
       <c r="F39">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G39">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H39">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I39">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="J39">
         <v>2</v>
       </c>
       <c r="K39" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L39">
-        <v>0.308</v>
+        <v>0.302</v>
       </c>
     </row>
     <row r="40" spans="1:12">
@@ -2164,37 +2167,37 @@
         <v>50</v>
       </c>
       <c r="B40" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C40" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="D40">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E40">
-        <v>668</v>
+        <v>5288</v>
       </c>
       <c r="F40">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G40">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H40">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="I40">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="J40">
         <v>2</v>
       </c>
       <c r="K40" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L40">
-        <v>0.42</v>
+        <v>0.609</v>
       </c>
     </row>
     <row r="41" spans="1:12">
@@ -2202,37 +2205,37 @@
         <v>51</v>
       </c>
       <c r="B41" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C41" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="D41">
-        <v>55</v>
+        <v>12</v>
       </c>
       <c r="E41">
-        <v>1079680</v>
+        <v>36922</v>
       </c>
       <c r="F41">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="G41">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="H41">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="I41">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="J41">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K41" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L41">
-        <v>336.452</v>
+        <v>8.368</v>
       </c>
     </row>
     <row r="42" spans="1:12">
@@ -2240,22 +2243,22 @@
         <v>52</v>
       </c>
       <c r="B42" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C42" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="D42">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="E42">
-        <v>96491</v>
+        <v>1302</v>
       </c>
       <c r="F42">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G42">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="H42">
         <v>2</v>
@@ -2267,10 +2270,10 @@
         <v>2</v>
       </c>
       <c r="K42" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L42">
-        <v>33.67</v>
+        <v>0.179</v>
       </c>
     </row>
     <row r="43" spans="1:12">
@@ -2278,37 +2281,37 @@
         <v>53</v>
       </c>
       <c r="B43" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C43" t="s">
+        <v>95</v>
+      </c>
+      <c r="D43">
+        <v>192</v>
+      </c>
+      <c r="E43">
+        <v>154899</v>
+      </c>
+      <c r="F43">
+        <v>54</v>
+      </c>
+      <c r="G43">
         <v>92</v>
       </c>
-      <c r="D43">
-        <v>16</v>
-      </c>
-      <c r="E43">
-        <v>6118</v>
-      </c>
-      <c r="F43">
-        <v>9</v>
-      </c>
-      <c r="G43">
-        <v>2</v>
-      </c>
       <c r="H43">
-        <v>3</v>
+        <v>20</v>
       </c>
       <c r="I43">
-        <v>3</v>
+        <v>39</v>
       </c>
       <c r="J43">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K43" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L43">
-        <v>2.908</v>
+        <v>40.634</v>
       </c>
     </row>
     <row r="44" spans="1:12">
@@ -2316,37 +2319,37 @@
         <v>54</v>
       </c>
       <c r="B44" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C44" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="D44">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E44">
-        <v>23</v>
+        <v>2735</v>
       </c>
       <c r="F44">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G44">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H44">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I44">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J44">
         <v>2</v>
       </c>
       <c r="K44" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L44">
-        <v>0.002</v>
+        <v>0.6830000000000001</v>
       </c>
     </row>
     <row r="45" spans="1:12">
@@ -2354,37 +2357,37 @@
         <v>55</v>
       </c>
       <c r="B45" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C45" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D45">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="E45">
-        <v>1249411</v>
+        <v>712</v>
       </c>
       <c r="F45">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G45">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="H45">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="I45">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J45">
         <v>2</v>
       </c>
       <c r="K45" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L45">
-        <v>114.714</v>
+        <v>0.091</v>
       </c>
     </row>
     <row r="46" spans="1:12">
@@ -2392,37 +2395,37 @@
         <v>56</v>
       </c>
       <c r="B46" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C46" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D46">
-        <v>25</v>
+        <v>8</v>
       </c>
       <c r="E46">
-        <v>5647694</v>
+        <v>81850</v>
       </c>
       <c r="F46">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="G46">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H46">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="I46">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J46">
         <v>2</v>
       </c>
       <c r="K46" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L46">
-        <v>857.134</v>
+        <v>22.794</v>
       </c>
     </row>
     <row r="47" spans="1:12">
@@ -2430,37 +2433,37 @@
         <v>57</v>
       </c>
       <c r="B47" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C47" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="D47">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="E47">
-        <v>4395</v>
+        <v>5751408</v>
       </c>
       <c r="F47">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="G47">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H47">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="I47">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="J47">
         <v>2</v>
       </c>
       <c r="K47" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L47">
-        <v>0.772</v>
+        <v>2058.564</v>
       </c>
     </row>
     <row r="48" spans="1:12">
@@ -2468,37 +2471,37 @@
         <v>58</v>
       </c>
       <c r="B48" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C48" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D48">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="E48">
-        <v>1754397</v>
+        <v>668</v>
       </c>
       <c r="F48">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="G48">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="H48">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="I48">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J48">
         <v>2</v>
       </c>
       <c r="K48" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L48">
-        <v>773.989</v>
+        <v>0.308</v>
       </c>
     </row>
     <row r="49" spans="1:12">
@@ -2506,37 +2509,37 @@
         <v>59</v>
       </c>
       <c r="B49" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C49" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="D49">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="E49">
-        <v>11150</v>
+        <v>668</v>
       </c>
       <c r="F49">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G49">
         <v>3</v>
       </c>
       <c r="H49">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I49">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J49">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K49" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L49">
-        <v>2.596</v>
+        <v>0.42</v>
       </c>
     </row>
     <row r="50" spans="1:12">
@@ -2544,37 +2547,37 @@
         <v>60</v>
       </c>
       <c r="B50" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C50" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="D50">
-        <v>15</v>
+        <v>55</v>
       </c>
       <c r="E50">
-        <v>10324</v>
+        <v>1079680</v>
       </c>
       <c r="F50">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="G50">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="H50">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="I50">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="J50">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K50" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L50">
-        <v>2.065</v>
+        <v>336.452</v>
       </c>
     </row>
     <row r="51" spans="1:12">
@@ -2582,37 +2585,37 @@
         <v>61</v>
       </c>
       <c r="B51" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C51" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D51">
-        <v>119</v>
+        <v>11</v>
       </c>
       <c r="E51">
-        <v>11004</v>
+        <v>96491</v>
       </c>
       <c r="F51">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G51">
-        <v>112</v>
+        <v>1</v>
       </c>
       <c r="H51">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I51">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J51">
         <v>2</v>
       </c>
       <c r="K51" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L51">
-        <v>1.833</v>
+        <v>33.67</v>
       </c>
     </row>
     <row r="52" spans="1:12">
@@ -2620,19 +2623,19 @@
         <v>62</v>
       </c>
       <c r="B52" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C52" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="D52">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="E52">
-        <v>19297</v>
+        <v>6118</v>
       </c>
       <c r="F52">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="G52">
         <v>2</v>
@@ -2644,13 +2647,13 @@
         <v>3</v>
       </c>
       <c r="J52">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K52" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L52">
-        <v>3.573</v>
+        <v>2.908</v>
       </c>
     </row>
     <row r="53" spans="1:12">
@@ -2658,37 +2661,37 @@
         <v>63</v>
       </c>
       <c r="B53" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C53" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="D53">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E53">
-        <v>83</v>
+        <v>23</v>
       </c>
       <c r="F53">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G53">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H53">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I53">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J53">
         <v>2</v>
       </c>
       <c r="K53" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L53">
-        <v>0.024</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="54" spans="1:12">
@@ -2696,37 +2699,37 @@
         <v>64</v>
       </c>
       <c r="B54" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C54" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="D54">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="E54">
-        <v>171</v>
+        <v>1249411</v>
       </c>
       <c r="F54">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G54">
         <v>9</v>
       </c>
       <c r="H54">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I54">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J54">
         <v>2</v>
       </c>
       <c r="K54" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L54">
-        <v>0.013</v>
+        <v>114.714</v>
       </c>
     </row>
     <row r="55" spans="1:12">
@@ -2734,37 +2737,37 @@
         <v>65</v>
       </c>
       <c r="B55" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C55" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="D55">
         <v>25</v>
       </c>
       <c r="E55">
-        <v>5302</v>
+        <v>5647694</v>
       </c>
       <c r="F55">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="G55">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="H55">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="I55">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="J55">
         <v>2</v>
       </c>
       <c r="K55" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L55">
-        <v>1.266</v>
+        <v>857.134</v>
       </c>
     </row>
     <row r="56" spans="1:12">
@@ -2772,29 +2775,29 @@
         <v>66</v>
       </c>
       <c r="B56" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C56" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="D56">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="E56">
-        <v>32231279</v>
+        <v>4395</v>
       </c>
       <c r="F56">
+        <v>9</v>
+      </c>
+      <c r="G56">
         <v>4</v>
       </c>
-      <c r="G56">
-        <v>2</v>
-      </c>
       <c r="H56">
+        <v>7</v>
+      </c>
+      <c r="I56">
         <v>6</v>
       </c>
-      <c r="I56">
-        <v>5</v>
-      </c>
       <c r="J56">
         <v>2</v>
       </c>
@@ -2802,7 +2805,7 @@
         <v>100</v>
       </c>
       <c r="L56">
-        <v>969.1849999999999</v>
+        <v>0.772</v>
       </c>
     </row>
     <row r="57" spans="1:12">
@@ -2810,28 +2813,28 @@
         <v>67</v>
       </c>
       <c r="B57" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C57" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="D57">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="E57">
-        <v>148021</v>
+        <v>1754397</v>
       </c>
       <c r="F57">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="G57">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="H57">
         <v>5</v>
       </c>
       <c r="I57">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J57">
         <v>2</v>
@@ -2840,7 +2843,7 @@
         <v>100</v>
       </c>
       <c r="L57">
-        <v>20.369</v>
+        <v>773.989</v>
       </c>
     </row>
     <row r="58" spans="1:12">
@@ -2848,28 +2851,28 @@
         <v>68</v>
       </c>
       <c r="B58" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C58" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="D58">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="E58">
-        <v>173933</v>
+        <v>11150</v>
       </c>
       <c r="F58">
         <v>4</v>
       </c>
       <c r="G58">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H58">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I58">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J58">
         <v>3</v>
@@ -2878,7 +2881,7 @@
         <v>100</v>
       </c>
       <c r="L58">
-        <v>40.435</v>
+        <v>2.596</v>
       </c>
     </row>
     <row r="59" spans="1:12">
@@ -2886,37 +2889,37 @@
         <v>69</v>
       </c>
       <c r="B59" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C59" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="D59">
         <v>15</v>
       </c>
       <c r="E59">
-        <v>15000713</v>
+        <v>10324</v>
       </c>
       <c r="F59">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G59">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="H59">
         <v>3</v>
       </c>
       <c r="I59">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J59">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K59" t="s">
         <v>100</v>
       </c>
       <c r="L59">
-        <v>10786.244</v>
+        <v>2.065</v>
       </c>
     </row>
     <row r="60" spans="1:12">
@@ -2924,28 +2927,28 @@
         <v>70</v>
       </c>
       <c r="B60" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C60" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="D60">
-        <v>21</v>
+        <v>119</v>
       </c>
       <c r="E60">
-        <v>2146112</v>
+        <v>11004</v>
       </c>
       <c r="F60">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G60">
-        <v>0</v>
+        <v>112</v>
       </c>
       <c r="H60">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="I60">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J60">
         <v>2</v>
@@ -2954,7 +2957,7 @@
         <v>100</v>
       </c>
       <c r="L60">
-        <v>523.1</v>
+        <v>1.833</v>
       </c>
     </row>
     <row r="61" spans="1:12">
@@ -2962,28 +2965,28 @@
         <v>71</v>
       </c>
       <c r="B61" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C61" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D61">
-        <v>42</v>
+        <v>12</v>
       </c>
       <c r="E61">
-        <v>20679117</v>
+        <v>19297</v>
       </c>
       <c r="F61">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="G61">
         <v>2</v>
       </c>
       <c r="H61">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="I61">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="J61">
         <v>3</v>
@@ -2992,7 +2995,7 @@
         <v>100</v>
       </c>
       <c r="L61">
-        <v>2754.622</v>
+        <v>3.573</v>
       </c>
     </row>
     <row r="62" spans="1:12">
@@ -3000,37 +3003,37 @@
         <v>72</v>
       </c>
       <c r="B62" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C62" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="D62">
-        <v>129</v>
+        <v>13</v>
       </c>
       <c r="E62">
-        <v>41328337</v>
+        <v>83</v>
       </c>
       <c r="F62">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="G62">
-        <v>102</v>
+        <v>4</v>
       </c>
       <c r="H62">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="I62">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="J62">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K62" t="s">
         <v>100</v>
       </c>
       <c r="L62">
-        <v>4578.511</v>
+        <v>0.024</v>
       </c>
     </row>
     <row r="63" spans="1:12">
@@ -3038,37 +3041,37 @@
         <v>73</v>
       </c>
       <c r="B63" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C63" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="D63">
-        <v>67</v>
+        <v>19</v>
       </c>
       <c r="E63">
-        <v>74063</v>
+        <v>171</v>
       </c>
       <c r="F63">
+        <v>1</v>
+      </c>
+      <c r="G63">
+        <v>9</v>
+      </c>
+      <c r="H63">
+        <v>5</v>
+      </c>
+      <c r="I63">
         <v>4</v>
       </c>
-      <c r="G63">
-        <v>21</v>
-      </c>
-      <c r="H63">
-        <v>9</v>
-      </c>
-      <c r="I63">
-        <v>13</v>
-      </c>
       <c r="J63">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K63" t="s">
         <v>100</v>
       </c>
       <c r="L63">
-        <v>10.695</v>
+        <v>0.013</v>
       </c>
     </row>
     <row r="64" spans="1:12">
@@ -3076,22 +3079,22 @@
         <v>74</v>
       </c>
       <c r="B64" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C64" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="D64">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="E64">
-        <v>16664809</v>
+        <v>5302</v>
       </c>
       <c r="F64">
-        <v>30</v>
+        <v>11</v>
       </c>
       <c r="G64">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="H64">
         <v>3</v>
@@ -3106,7 +3109,7 @@
         <v>100</v>
       </c>
       <c r="L64">
-        <v>2008.983</v>
+        <v>1.266</v>
       </c>
     </row>
     <row r="65" spans="1:12">
@@ -3114,37 +3117,37 @@
         <v>75</v>
       </c>
       <c r="B65" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C65" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="D65">
-        <v>221</v>
+        <v>19</v>
       </c>
       <c r="E65">
-        <v>13787005</v>
+        <v>32231279</v>
       </c>
       <c r="F65">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="G65">
-        <v>40</v>
+        <v>2</v>
       </c>
       <c r="H65">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="I65">
-        <v>21</v>
+        <v>5</v>
       </c>
       <c r="J65">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="K65" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="L65">
-        <v>9343.481</v>
+        <v>969.1849999999999</v>
       </c>
     </row>
     <row r="66" spans="1:12">
@@ -3152,37 +3155,37 @@
         <v>76</v>
       </c>
       <c r="B66" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C66" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D66">
-        <v>31</v>
+        <v>15</v>
       </c>
       <c r="E66">
-        <v>4257145</v>
+        <v>148021</v>
       </c>
       <c r="F66">
-        <v>17</v>
+        <v>5</v>
       </c>
       <c r="G66">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H66">
+        <v>5</v>
+      </c>
+      <c r="I66">
         <v>4</v>
       </c>
-      <c r="I66">
-        <v>6</v>
-      </c>
       <c r="J66">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K66" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="L66">
-        <v>748.396</v>
+        <v>20.369</v>
       </c>
     </row>
     <row r="67" spans="1:12">
@@ -3190,37 +3193,37 @@
         <v>77</v>
       </c>
       <c r="B67" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C67" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D67">
-        <v>51</v>
+        <v>12</v>
       </c>
       <c r="E67">
-        <v>4247264</v>
+        <v>173933</v>
       </c>
       <c r="F67">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="G67">
         <v>0</v>
       </c>
       <c r="H67">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="I67">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="J67">
         <v>3</v>
       </c>
       <c r="K67" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="L67">
-        <v>2679.668</v>
+        <v>40.435</v>
       </c>
     </row>
     <row r="68" spans="1:12">
@@ -3228,37 +3231,37 @@
         <v>78</v>
       </c>
       <c r="B68" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C68" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="D68">
-        <v>140</v>
+        <v>15</v>
       </c>
       <c r="E68">
-        <v>5434924</v>
+        <v>15000713</v>
       </c>
       <c r="F68">
-        <v>51</v>
+        <v>4</v>
       </c>
       <c r="G68">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="H68">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="I68">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="J68">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K68" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="L68">
-        <v>3006.228</v>
+        <v>10786.244</v>
       </c>
     </row>
     <row r="69" spans="1:12">
@@ -3266,37 +3269,37 @@
         <v>79</v>
       </c>
       <c r="B69" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C69" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="D69">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="E69">
-        <v>1018324</v>
+        <v>2146112</v>
       </c>
       <c r="F69">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G69">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="H69">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="I69">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="J69">
         <v>2</v>
       </c>
       <c r="K69" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="L69">
-        <v>184.365</v>
+        <v>523.1</v>
       </c>
     </row>
     <row r="70" spans="1:12">
@@ -3304,37 +3307,37 @@
         <v>80</v>
       </c>
       <c r="B70" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C70" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="D70">
-        <v>20</v>
+        <v>42</v>
       </c>
       <c r="E70">
-        <v>429805</v>
+        <v>20679117</v>
       </c>
       <c r="F70">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="G70">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="H70">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="I70">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="J70">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K70" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="L70">
-        <v>40</v>
+        <v>2754.622</v>
       </c>
     </row>
     <row r="71" spans="1:12">
@@ -3348,31 +3351,31 @@
         <v>96</v>
       </c>
       <c r="D71">
-        <v>15</v>
+        <v>129</v>
       </c>
       <c r="E71">
-        <v>32561</v>
+        <v>41328337</v>
       </c>
       <c r="F71">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G71">
-        <v>6</v>
+        <v>102</v>
       </c>
       <c r="H71">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="I71">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="J71">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K71" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="L71">
-        <v>20.848</v>
+        <v>4578.511</v>
       </c>
     </row>
     <row r="72" spans="1:12">
@@ -3383,34 +3386,34 @@
         <v>91</v>
       </c>
       <c r="C72" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="D72">
-        <v>37</v>
+        <v>67</v>
       </c>
       <c r="E72">
-        <v>20000</v>
+        <v>74063</v>
       </c>
       <c r="F72">
-        <v>37</v>
+        <v>4</v>
       </c>
       <c r="G72">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="H72">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="I72">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="J72">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K72" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="L72">
-        <v>33.428</v>
+        <v>10.695</v>
       </c>
     </row>
     <row r="73" spans="1:12">
@@ -3421,34 +3424,34 @@
         <v>91</v>
       </c>
       <c r="C73" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D73">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="E73">
-        <v>299285</v>
+        <v>16664809</v>
       </c>
       <c r="F73">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G73">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="H73">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I73">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J73">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K73" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="L73">
-        <v>647.349</v>
+        <v>2008.983</v>
       </c>
     </row>
     <row r="74" spans="1:12">
@@ -3459,34 +3462,34 @@
         <v>91</v>
       </c>
       <c r="C74" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D74">
-        <v>20</v>
+        <v>221</v>
       </c>
       <c r="E74">
-        <v>20000</v>
+        <v>13787005</v>
       </c>
       <c r="F74">
-        <v>20</v>
+        <v>69</v>
       </c>
       <c r="G74">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="H74">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="I74">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="J74">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="K74" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="L74">
-        <v>24.462</v>
+        <v>9343.481</v>
       </c>
     </row>
     <row r="75" spans="1:12">
@@ -3497,34 +3500,34 @@
         <v>91</v>
       </c>
       <c r="C75" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D75">
-        <v>55</v>
+        <v>31</v>
       </c>
       <c r="E75">
-        <v>581012</v>
+        <v>4257145</v>
       </c>
       <c r="F75">
-        <v>1</v>
+        <v>17</v>
       </c>
       <c r="G75">
-        <v>54</v>
+        <v>0</v>
       </c>
       <c r="H75">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I75">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="J75">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K75" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="L75">
-        <v>255.645</v>
+        <v>748.396</v>
       </c>
     </row>
     <row r="76" spans="1:12">
@@ -3535,34 +3538,34 @@
         <v>91</v>
       </c>
       <c r="C76" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="D76">
-        <v>25</v>
+        <v>51</v>
       </c>
       <c r="E76">
-        <v>1000</v>
+        <v>4247264</v>
       </c>
       <c r="F76">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="G76">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="H76">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="I76">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J76">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K76" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="L76">
-        <v>0.444</v>
+        <v>2679.668</v>
       </c>
     </row>
     <row r="77" spans="1:12">
@@ -3573,34 +3576,34 @@
         <v>91</v>
       </c>
       <c r="C77" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="D77">
-        <v>27</v>
+        <v>140</v>
       </c>
       <c r="E77">
-        <v>20000</v>
+        <v>5434924</v>
       </c>
       <c r="F77">
-        <v>27</v>
+        <v>51</v>
       </c>
       <c r="G77">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="H77">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="I77">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="J77">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K77" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="L77">
-        <v>24.82</v>
+        <v>3006.228</v>
       </c>
     </row>
     <row r="78" spans="1:12">
@@ -3614,31 +3617,31 @@
         <v>96</v>
       </c>
       <c r="D78">
-        <v>41</v>
+        <v>19</v>
       </c>
       <c r="E78">
-        <v>494021</v>
+        <v>1018324</v>
       </c>
       <c r="F78">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G78">
-        <v>37</v>
+        <v>10</v>
       </c>
       <c r="H78">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I78">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J78">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K78" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="L78">
-        <v>266.086</v>
+        <v>184.365</v>
       </c>
     </row>
     <row r="79" spans="1:12">
@@ -3652,31 +3655,31 @@
         <v>96</v>
       </c>
       <c r="D79">
-        <v>59</v>
+        <v>20</v>
       </c>
       <c r="E79">
-        <v>39644</v>
+        <v>429805</v>
       </c>
       <c r="F79">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G79">
-        <v>59</v>
+        <v>12</v>
       </c>
       <c r="H79">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I79">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J79">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K79" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="L79">
-        <v>18.712</v>
+        <v>40</v>
       </c>
     </row>
   </sheetData>

</xml_diff>